<commit_message>
Update tax invoice template
</commit_message>
<xml_diff>
--- a/vba/税务局发票模版.xlsx
+++ b/vba/税务局发票模版.xlsx
@@ -124,30 +124,7 @@
     <t>合计</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <rFont val="宋体"/>
-        <charset val="134"/>
-      </rPr>
-      <t>TOTAL QUANTITY:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <rFont val="宋体"/>
-        <charset val="134"/>
-      </rPr>
-      <t>1</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <rFont val="宋体"/>
-        <charset val="134"/>
-      </rPr>
-      <t xml:space="preserve">                   </t>
-    </r>
+    <t xml:space="preserve">TOTAL QUANTITY:1                   </t>
   </si>
   <si>
     <t>总量：1</t>
@@ -311,7 +288,7 @@
     <numFmt numFmtId="179" formatCode="0.00_);[Red]\(0.00\)"/>
     <numFmt numFmtId="180" formatCode="0.00_ "/>
   </numFmts>
-  <fonts count="50">
+  <fonts count="57">
     <font>
       <sz val="12"/>
       <name val="宋体"/>
@@ -439,6 +416,38 @@
     <font>
       <u/>
       <sz val="12"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+    </font>
+    <font>
+      <sz val="13"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="1"/>
       <name val="宋体"/>
       <charset val="134"/>
     </font>
@@ -450,53 +459,69 @@
       <charset val="0"/>
     </font>
     <font>
+      <b/>
+      <sz val="16"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="隶书"/>
+      <charset val="0"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+    </font>
+    <font>
       <u/>
       <sz val="12"/>
       <color indexed="12"/>
       <name val="新細明體"/>
       <charset val="0"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color rgb="FFFF0000"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Times New Roman"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color indexed="8"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="12"/>
-      <color indexed="10"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="宋体"/>
-      <charset val="134"/>
     </font>
     <font>
       <u/>
@@ -971,140 +996,140 @@
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="top"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="top"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="3" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="40" fillId="4" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="4" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="42" fillId="5" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="43" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="44" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="45" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="46" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="47" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="48" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="49" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="49" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="48" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="48" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="49" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="49" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="48" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="48" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="49" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="49" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="48" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="48" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="49" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="49" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="48" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="48" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="49" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="49" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="48" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="48" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="49" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="49" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="48" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="40" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="45" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="45" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="46" fillId="3" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="4" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="48" fillId="4" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="49" fillId="5" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="51" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="52" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="53" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="54" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="55" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="56" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="56" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="55" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="55" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="56" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="56" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="55" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="55" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="56" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="56" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="55" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="55" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="56" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="56" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="55" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="55" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="56" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="56" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="55" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="55" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="56" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="56" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="55" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="83">
+  <cellXfs count="94">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -1204,80 +1229,101 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="177" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="6" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="6" applyFill="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="6" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="6" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="29" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="30" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="49" fontId="25" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="31" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="24" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="176" fontId="25" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="14" fontId="25" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="178" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="178" fontId="34" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="179" fontId="30" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="179" fontId="32" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="180" fontId="25" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="50">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -1637,366 +1683,366 @@
   <dimension ref="A1:K29"/>
   <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="17.6"/>
   <cols>
-    <col min="1" max="1" width="13.0803571428571" style="5" customWidth="1"/>
-    <col min="2" max="2" width="4.41071428571429" style="5" customWidth="1"/>
-    <col min="3" max="3" width="18.5" style="5" customWidth="1"/>
-    <col min="4" max="4" width="9.33035714285714" style="5" customWidth="1"/>
-    <col min="5" max="5" width="16.5803571428571" style="5" customWidth="1"/>
-    <col min="6" max="6" width="15.8303571428571" style="5" customWidth="1"/>
-    <col min="7" max="7" width="16.5" style="5" customWidth="1"/>
-    <col min="8" max="8" width="9.5" style="5"/>
-    <col min="9" max="34" width="9" style="5"/>
-    <col min="35" max="16384" width="8.66071428571429" style="5"/>
+    <col min="1" max="1" width="13.0803571428571" style="51" customWidth="1"/>
+    <col min="2" max="2" width="4.41071428571429" style="51" customWidth="1"/>
+    <col min="3" max="3" width="18.5" style="51" customWidth="1"/>
+    <col min="4" max="4" width="9.33035714285714" style="51" customWidth="1"/>
+    <col min="5" max="5" width="16.5803571428571" style="51" customWidth="1"/>
+    <col min="6" max="6" width="15.8303571428571" style="51" customWidth="1"/>
+    <col min="7" max="7" width="16.5" style="51" customWidth="1"/>
+    <col min="8" max="8" width="9.5" style="51"/>
+    <col min="9" max="34" width="9" style="51"/>
+    <col min="35" max="16384" width="8.66071428571429" style="51"/>
   </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1" ht="29.25" customHeight="1" spans="1:10">
-      <c r="A1" s="8"/>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8" t="s">
+    <row r="1" s="49" customFormat="1" ht="29.25" customHeight="1" spans="1:10">
+      <c r="A1" s="52"/>
+      <c r="B1" s="52"/>
+      <c r="C1" s="52"/>
+      <c r="D1" s="52"/>
+      <c r="E1" s="52" t="s">
         <v>0</v>
       </c>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8"/>
-      <c r="H1" s="8"/>
-      <c r="I1" s="35"/>
-      <c r="J1" s="35"/>
+      <c r="F1" s="52"/>
+      <c r="G1" s="52"/>
+      <c r="H1" s="52"/>
+      <c r="I1" s="86"/>
+      <c r="J1" s="86"/>
     </row>
     <row r="2" ht="28.5" customHeight="1" spans="1:9">
-      <c r="A2" s="9" t="s">
+      <c r="A2" s="53" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="9"/>
-      <c r="C2" s="9"/>
-      <c r="D2" s="9"/>
-      <c r="E2" s="9"/>
-      <c r="F2" s="9"/>
-      <c r="G2" s="9"/>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
+      <c r="B2" s="53"/>
+      <c r="C2" s="53"/>
+      <c r="D2" s="53"/>
+      <c r="E2" s="53"/>
+      <c r="F2" s="53"/>
+      <c r="G2" s="53"/>
+      <c r="H2" s="50"/>
+      <c r="I2" s="50"/>
     </row>
     <row r="3" ht="22.5" customHeight="1" spans="1:9">
-      <c r="A3" s="9"/>
-      <c r="B3" s="9"/>
-      <c r="C3" s="9"/>
-      <c r="D3" s="9"/>
-      <c r="E3" s="9"/>
-      <c r="F3" s="9"/>
-      <c r="G3" s="9"/>
-      <c r="H3" s="2"/>
-      <c r="I3" s="2"/>
+      <c r="A3" s="53"/>
+      <c r="B3" s="53"/>
+      <c r="C3" s="53"/>
+      <c r="D3" s="53"/>
+      <c r="E3" s="53"/>
+      <c r="F3" s="53"/>
+      <c r="G3" s="53"/>
+      <c r="H3" s="50"/>
+      <c r="I3" s="50"/>
     </row>
     <row r="4" ht="17.25" customHeight="1" spans="1:9">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="50" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="2"/>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2"/>
-      <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
-      <c r="I4" s="2"/>
+      <c r="B4" s="50"/>
+      <c r="C4" s="50"/>
+      <c r="D4" s="50"/>
+      <c r="E4" s="50"/>
+      <c r="F4" s="50"/>
+      <c r="G4" s="50"/>
+      <c r="H4" s="50"/>
+      <c r="I4" s="50"/>
     </row>
     <row r="5" ht="17.25" customHeight="1" spans="1:9">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="50" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="2"/>
-      <c r="C5" s="2"/>
-      <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
-      <c r="F5" s="2"/>
-      <c r="G5" s="2"/>
-      <c r="H5" s="2"/>
-      <c r="I5" s="2"/>
-    </row>
-    <row r="6" s="2" customFormat="1" ht="17.25" customHeight="1" spans="1:8">
-      <c r="A6" s="49" t="s">
+      <c r="B5" s="50"/>
+      <c r="C5" s="50"/>
+      <c r="D5" s="50"/>
+      <c r="E5" s="50"/>
+      <c r="F5" s="50"/>
+      <c r="G5" s="50"/>
+      <c r="H5" s="50"/>
+      <c r="I5" s="50"/>
+    </row>
+    <row r="6" s="50" customFormat="1" ht="17.25" customHeight="1" spans="1:8">
+      <c r="A6" s="54" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="50"/>
-      <c r="G6" s="37"/>
-      <c r="H6" s="37"/>
+      <c r="B6" s="55"/>
+      <c r="G6" s="81"/>
+      <c r="H6" s="81"/>
     </row>
     <row r="7" spans="1:1">
-      <c r="A7" s="5" t="s">
+      <c r="A7" s="56" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="8" ht="23.2" spans="1:11">
-      <c r="A8" s="51" t="s">
+      <c r="A8" s="57" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="51"/>
-      <c r="C8" s="52"/>
-      <c r="D8" s="52"/>
-      <c r="E8" s="52"/>
-      <c r="F8" s="52"/>
-      <c r="G8" s="52"/>
-      <c r="H8" s="12"/>
-      <c r="I8" s="12"/>
-      <c r="J8" s="12"/>
-      <c r="K8" s="12"/>
+      <c r="B8" s="57"/>
+      <c r="C8" s="58"/>
+      <c r="D8" s="58"/>
+      <c r="E8" s="58"/>
+      <c r="F8" s="58"/>
+      <c r="G8" s="58"/>
+      <c r="H8" s="82"/>
+      <c r="I8" s="82"/>
+      <c r="J8" s="82"/>
+      <c r="K8" s="82"/>
     </row>
     <row r="9" ht="23.2" spans="1:11">
-      <c r="A9" s="53" t="s">
+      <c r="A9" s="59" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="53"/>
-      <c r="C9" s="54"/>
-      <c r="D9" s="54"/>
-      <c r="E9" s="54"/>
-      <c r="F9" s="54"/>
-      <c r="G9" s="54"/>
-      <c r="H9" s="12"/>
-      <c r="I9" s="12"/>
-      <c r="J9" s="12"/>
-      <c r="K9" s="12"/>
+      <c r="B9" s="59"/>
+      <c r="C9" s="60"/>
+      <c r="D9" s="60"/>
+      <c r="E9" s="60"/>
+      <c r="F9" s="60"/>
+      <c r="G9" s="60"/>
+      <c r="H9" s="82"/>
+      <c r="I9" s="82"/>
+      <c r="J9" s="82"/>
+      <c r="K9" s="82"/>
     </row>
     <row r="11" ht="21.75" customHeight="1" spans="1:7">
-      <c r="A11" s="55" t="s">
+      <c r="A11" s="56" t="s">
         <v>8</v>
       </c>
-      <c r="B11" s="56"/>
-      <c r="C11" s="13" t="s">
+      <c r="B11" s="61"/>
+      <c r="C11" s="62" t="s">
         <v>9</v>
       </c>
-      <c r="D11" s="57"/>
-      <c r="E11" s="71" t="s">
+      <c r="D11" s="63"/>
+      <c r="E11" s="83" t="s">
         <v>10</v>
       </c>
-      <c r="F11" s="72"/>
-      <c r="G11" s="73"/>
+      <c r="F11" s="84"/>
+      <c r="G11" s="85"/>
     </row>
     <row r="12" ht="21.75" customHeight="1" spans="1:7">
-      <c r="A12" s="55" t="s">
+      <c r="A12" s="56" t="s">
         <v>11</v>
       </c>
-      <c r="B12" s="56"/>
-      <c r="C12" s="58" t="s">
+      <c r="B12" s="61"/>
+      <c r="C12" s="63" t="s">
         <v>12</v>
       </c>
-      <c r="D12" s="57"/>
-      <c r="E12" s="55" t="s">
+      <c r="D12" s="63"/>
+      <c r="E12" s="56" t="s">
         <v>13</v>
       </c>
-      <c r="F12" s="72"/>
-      <c r="G12" s="73"/>
-    </row>
-    <row r="13" s="3" customFormat="1" ht="21" customHeight="1" spans="1:10">
-      <c r="A13" s="59" t="s">
+      <c r="F12" s="84"/>
+      <c r="G12" s="85"/>
+    </row>
+    <row r="13" s="49" customFormat="1" ht="21" customHeight="1" spans="1:10">
+      <c r="A13" s="64" t="s">
         <v>14</v>
       </c>
-      <c r="B13" s="59"/>
-      <c r="C13" s="60"/>
-      <c r="D13" s="61"/>
-      <c r="E13" s="60"/>
-      <c r="F13" s="60"/>
-      <c r="G13" s="74"/>
-      <c r="H13" s="74"/>
-      <c r="I13" s="74"/>
-      <c r="J13" s="74"/>
-    </row>
-    <row r="14" s="3" customFormat="1" ht="21" customHeight="1" spans="1:10">
-      <c r="A14" s="62" t="s">
+      <c r="B13" s="64"/>
+      <c r="C13" s="65"/>
+      <c r="D13" s="65"/>
+      <c r="E13" s="65"/>
+      <c r="F13" s="65"/>
+      <c r="G13" s="86"/>
+      <c r="H13" s="86"/>
+      <c r="I13" s="86"/>
+      <c r="J13" s="86"/>
+    </row>
+    <row r="14" s="49" customFormat="1" ht="21" customHeight="1" spans="1:10">
+      <c r="A14" s="66" t="s">
         <v>15</v>
       </c>
-      <c r="B14" s="63"/>
-      <c r="C14" s="61"/>
-      <c r="D14" s="61"/>
-      <c r="E14" s="60"/>
-      <c r="F14" s="60"/>
-      <c r="G14" s="74"/>
-      <c r="H14" s="74"/>
-      <c r="I14" s="74"/>
-      <c r="J14" s="74"/>
+      <c r="B14" s="66"/>
+      <c r="C14" s="65"/>
+      <c r="D14" s="65"/>
+      <c r="E14" s="65"/>
+      <c r="F14" s="65"/>
+      <c r="G14" s="86"/>
+      <c r="H14" s="86"/>
+      <c r="I14" s="86"/>
+      <c r="J14" s="86"/>
     </row>
     <row r="15" ht="19.2" spans="1:8">
-      <c r="A15" s="2"/>
-      <c r="B15" s="2"/>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
-      <c r="F15" s="2"/>
-      <c r="G15" s="2"/>
-      <c r="H15" s="2"/>
+      <c r="A15" s="50"/>
+      <c r="B15" s="50"/>
+      <c r="C15" s="50"/>
+      <c r="D15" s="50"/>
+      <c r="E15" s="50"/>
+      <c r="F15" s="50"/>
+      <c r="G15" s="50"/>
+      <c r="H15" s="50"/>
     </row>
     <row r="16" ht="19.2" spans="1:8">
-      <c r="A16" s="18" t="s">
+      <c r="A16" s="50" t="s">
         <v>16</v>
       </c>
-      <c r="B16" s="18"/>
-      <c r="C16" s="2"/>
-      <c r="D16" s="2"/>
-      <c r="E16" s="2"/>
-      <c r="F16" s="2" t="s">
+      <c r="B16" s="50"/>
+      <c r="C16" s="50"/>
+      <c r="D16" s="50"/>
+      <c r="E16" s="50"/>
+      <c r="F16" s="50" t="s">
         <v>17</v>
       </c>
-      <c r="G16" s="2"/>
-      <c r="H16" s="2"/>
+      <c r="G16" s="50"/>
+      <c r="H16" s="50"/>
     </row>
     <row r="17" ht="19.95" spans="1:8">
-      <c r="A17" s="18" t="s">
+      <c r="A17" s="50" t="s">
         <v>18</v>
       </c>
-      <c r="B17" s="18"/>
-      <c r="C17" s="2"/>
-      <c r="D17" s="2"/>
-      <c r="E17" s="2"/>
-      <c r="F17" s="2"/>
-      <c r="G17" s="2"/>
-      <c r="H17" s="2"/>
+      <c r="B17" s="50"/>
+      <c r="C17" s="50"/>
+      <c r="D17" s="50"/>
+      <c r="E17" s="50"/>
+      <c r="F17" s="50"/>
+      <c r="G17" s="50"/>
+      <c r="H17" s="50"/>
     </row>
     <row r="18" ht="45.75" customHeight="1" spans="1:7">
-      <c r="A18" s="64" t="s">
+      <c r="A18" s="67" t="s">
         <v>19</v>
       </c>
-      <c r="B18" s="64"/>
-      <c r="C18" s="64" t="s">
+      <c r="B18" s="68"/>
+      <c r="C18" s="67" t="s">
         <v>20</v>
       </c>
-      <c r="D18" s="64"/>
-      <c r="E18" s="75" t="s">
+      <c r="D18" s="68"/>
+      <c r="E18" s="67" t="s">
         <v>21</v>
       </c>
-      <c r="F18" s="75" t="s">
+      <c r="F18" s="67" t="s">
         <v>22</v>
       </c>
-      <c r="G18" s="64" t="s">
+      <c r="G18" s="67" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="19" ht="18.35" spans="1:7">
-      <c r="A19" s="24" t="s">
+      <c r="A19" s="69" t="s">
         <v>24</v>
       </c>
-      <c r="B19" s="24"/>
-      <c r="C19" s="29" t="s">
+      <c r="B19" s="69"/>
+      <c r="C19" s="70" t="s">
         <v>25</v>
       </c>
-      <c r="D19" s="29"/>
-      <c r="E19" s="29">
+      <c r="D19" s="70"/>
+      <c r="E19" s="70">
         <v>1</v>
       </c>
-      <c r="F19" s="76">
+      <c r="F19" s="87">
         <v>2405</v>
       </c>
-      <c r="G19" s="76">
+      <c r="G19" s="87">
         <f>F19</f>
         <v>2405</v>
       </c>
     </row>
     <row r="20" spans="1:7">
-      <c r="A20" s="24" t="s">
+      <c r="A20" s="69" t="s">
         <v>26</v>
       </c>
-      <c r="B20" s="24"/>
-      <c r="C20" s="30"/>
-      <c r="D20" s="30"/>
-      <c r="E20" s="29"/>
-      <c r="F20" s="77"/>
-      <c r="G20" s="77"/>
+      <c r="B20" s="69"/>
+      <c r="C20" s="71"/>
+      <c r="D20" s="71"/>
+      <c r="E20" s="70"/>
+      <c r="F20" s="87"/>
+      <c r="G20" s="87"/>
     </row>
     <row r="21" ht="18.35" spans="1:7">
-      <c r="A21" s="24" t="s">
+      <c r="A21" s="69" t="s">
         <v>27</v>
       </c>
-      <c r="B21" s="24"/>
-      <c r="C21" s="30"/>
-      <c r="D21" s="30"/>
-      <c r="E21" s="29"/>
-      <c r="F21" s="77"/>
-      <c r="G21" s="77"/>
+      <c r="B21" s="69"/>
+      <c r="C21" s="71"/>
+      <c r="D21" s="71"/>
+      <c r="E21" s="70"/>
+      <c r="F21" s="87"/>
+      <c r="G21" s="87"/>
     </row>
     <row r="22" ht="19.1" spans="1:8">
-      <c r="A22" s="65" t="s">
+      <c r="A22" s="72" t="s">
         <v>28</v>
       </c>
-      <c r="B22" s="65"/>
-      <c r="C22" s="66"/>
-      <c r="D22" s="66"/>
-      <c r="E22" s="66">
+      <c r="B22" s="73"/>
+      <c r="C22" s="74"/>
+      <c r="D22" s="74"/>
+      <c r="E22" s="74">
         <f>SUM(E19:E21)</f>
         <v>1</v>
       </c>
-      <c r="F22" s="66"/>
-      <c r="G22" s="78">
+      <c r="F22" s="74"/>
+      <c r="G22" s="88">
         <f>SUM(G19:G21)</f>
         <v>2405</v>
       </c>
-      <c r="H22" s="26"/>
+      <c r="H22" s="80"/>
     </row>
     <row r="23" ht="19.1" spans="1:8">
-      <c r="A23" s="67" t="s">
+      <c r="A23" s="75" t="s">
         <v>29</v>
       </c>
-      <c r="B23" s="67"/>
-      <c r="C23" s="68"/>
-      <c r="D23" s="68"/>
-      <c r="E23" s="66">
+      <c r="B23" s="76"/>
+      <c r="C23" s="77"/>
+      <c r="D23" s="77"/>
+      <c r="E23" s="74">
         <f>SUM(E20:E22)</f>
         <v>1</v>
       </c>
-      <c r="F23" s="66"/>
-      <c r="G23" s="78">
+      <c r="F23" s="74"/>
+      <c r="G23" s="88">
         <f>SUM(G20:G22)</f>
         <v>2405</v>
       </c>
-      <c r="H23" s="26"/>
+      <c r="H23" s="80"/>
     </row>
     <row r="24" ht="24" customHeight="1" spans="1:7">
-      <c r="A24" s="69" t="s">
+      <c r="A24" s="78" t="s">
         <v>30</v>
       </c>
-      <c r="B24" s="69"/>
-      <c r="C24" s="70"/>
-      <c r="D24" s="70"/>
-      <c r="E24" s="70"/>
-      <c r="F24" s="70"/>
-      <c r="G24" s="70"/>
+      <c r="B24" s="78"/>
+      <c r="C24" s="79"/>
+      <c r="D24" s="79"/>
+      <c r="E24" s="79"/>
+      <c r="F24" s="79"/>
+      <c r="G24" s="79"/>
     </row>
     <row r="25" spans="1:2">
-      <c r="A25" s="55" t="s">
+      <c r="A25" s="56" t="s">
         <v>31</v>
       </c>
-      <c r="B25" s="55"/>
+      <c r="B25" s="56"/>
     </row>
     <row r="26" spans="1:7">
-      <c r="A26" s="5" t="s">
+      <c r="A26" s="56" t="s">
         <v>32</v>
       </c>
-      <c r="F26" s="79" t="s">
+      <c r="F26" s="89" t="s">
         <v>33</v>
       </c>
-      <c r="G26" s="80"/>
+      <c r="G26" s="90"/>
     </row>
     <row r="27" spans="5:7">
-      <c r="E27" s="81" t="s">
+      <c r="E27" s="91" t="s">
         <v>34</v>
       </c>
-      <c r="F27" s="79"/>
-      <c r="G27" s="80"/>
+      <c r="F27" s="89"/>
+      <c r="G27" s="90"/>
     </row>
     <row r="28" ht="18.75" customHeight="1" spans="5:9">
-      <c r="E28" s="82" t="s">
+      <c r="E28" s="92" t="s">
         <v>35</v>
       </c>
-      <c r="F28" s="82"/>
-      <c r="G28" s="82"/>
-      <c r="H28" s="82"/>
-      <c r="I28" s="82"/>
+      <c r="F28" s="93"/>
+      <c r="G28" s="93"/>
+      <c r="H28" s="93"/>
+      <c r="I28" s="93"/>
     </row>
     <row r="29" spans="1:7">
-      <c r="A29" s="26"/>
-      <c r="B29" s="26"/>
-      <c r="C29" s="26"/>
-      <c r="D29" s="26"/>
-      <c r="E29" s="26"/>
-      <c r="F29" s="26"/>
-      <c r="G29" s="26"/>
+      <c r="A29" s="80"/>
+      <c r="B29" s="80"/>
+      <c r="C29" s="80"/>
+      <c r="D29" s="80"/>
+      <c r="E29" s="80"/>
+      <c r="F29" s="80"/>
+      <c r="G29" s="80"/>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>